<commit_message>
update results and figures
</commit_message>
<xml_diff>
--- a/result/case/case3.xlsx
+++ b/result/case/case3.xlsx
@@ -391,10 +391,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.2181795918367347</v>
+        <v>0.2439832341806382</v>
       </c>
       <c r="D2">
-        <v>4.990672434241546E-48</v>
+        <v>1.896606261923489E-17</v>
       </c>
     </row>
     <row r="3">
@@ -409,10 +409,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.1876816326530612</v>
+        <v>0.2071727961060033</v>
       </c>
       <c r="D3">
-        <v>7.390330900445726E-67</v>
+        <v>1.371208579800059E-25</v>
       </c>
     </row>
     <row r="4">
@@ -427,10 +427,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.3869142857142857</v>
+        <v>0.4304691725256896</v>
       </c>
       <c r="D4">
-        <v>1.716557997522749E-06</v>
+        <v>0.04764654115079872</v>
       </c>
     </row>
     <row r="5">
@@ -445,10 +445,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.3799673469387755</v>
+        <v>0.4326325040562466</v>
       </c>
       <c r="D5">
-        <v>3.234267975195473E-07</v>
+        <v>0.05583347285484098</v>
       </c>
     </row>
     <row r="6">
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.3206775510204082</v>
+        <v>0.3261898323418064</v>
       </c>
       <c r="D6">
-        <v>1.429894972415768E-15</v>
+        <v>1.470219394014243E-07</v>
       </c>
     </row>
     <row r="7">
@@ -481,10 +481,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.292669387755102</v>
+        <v>0.2761289886425095</v>
       </c>
       <c r="D7">
-        <v>2.796328581440632E-21</v>
+        <v>5.22770828231353E-13</v>
       </c>
     </row>
   </sheetData>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.5127123623584123</v>
+        <v>0.8276760656389834</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.4407668662231769</v>
+        <v>0.7957231689455366</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.3467850703613701</v>
+        <v>0.707747799985694</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.3345758759930962</v>
+        <v>0.6484832421018795</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.4617923319911552</v>
+        <v>0.7619731473471065</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.4242145571475958</v>
+        <v>0.7994555462466125</v>
       </c>
       <c r="D7">
         <v>0</v>

</xml_diff>